<commit_message>
feat: snapshot Q3 pricing, AI cloud settlement, Agent methodology, and weekly notes
Consolidate customer cloud settlement (incl. Tencent Sep), refresh commercial quotes and live price intermediates, add pricing human-interrupt tooling, and land Agent/GEO docs plus W39–W40 notes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/AI云业务/腾讯云对账/BID/腾讯云_服务费结算.xlsx
+++ b/AI云业务/腾讯云对账/BID/腾讯云_服务费结算.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -584,28 +584,60 @@
       <c r="H4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>BID账号</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>142932.83</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>2858.66</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>145791.49</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>真实消耗已预充值</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="6" t="n">
-        <v>322431.86</v>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="6" t="n">
+        <v>465364.69</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n">
-        <v>6448.64</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>328880.5</v>
-      </c>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr"/>
+      <c r="E6" s="6" t="n">
+        <v>9307.299999999999</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>474671.99</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>